<commit_message>
Fix import dedupe, transfers, categories, and learning from QA
Use per-source occurrence matching for overlapping statements, restore
app CSV round-trip dedupe, tighten card autopay detection on compact bank
text, default bank rows to Other with keyword guesses, and only persist
import rules after explicit review edits.

Co-authored-by: nixcapital <nixcapital@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/sample-bank.xlsx
+++ b/test/fixtures/sample-bank.xlsx
@@ -112,7 +112,7 @@
       <c r="C4"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CHASE CREDIT CRD AUTOPAY</t>
+          <t>XXXXX CREDIT CRDAUTOPAY   PPD</t>
         </is>
       </c>
       <c r="E4">
@@ -136,11 +136,11 @@
       <c r="C5"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Service Charge</t>
+          <t>STUDENT LOAN PAYMENT</t>
         </is>
       </c>
       <c r="E5">
-        <v>12</v>
+        <v>180</v>
       </c>
       <c r="F5"/>
       <c r="G5" t="inlineStr">
@@ -160,20 +160,20 @@
       <c r="C6"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COFFEE SHOP DOWNTOWN</t>
+          <t>Service Charge</t>
         </is>
       </c>
       <c r="E6">
-        <v>5.25</v>
+        <v>12</v>
       </c>
       <c r="F6"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Posted</t>
         </is>
       </c>
       <c r="H6">
-        <v>1291.56</v>
+        <v>1279.56</v>
       </c>
     </row>
     <row r="7">
@@ -184,23 +184,46 @@
       <c r="C7"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>WHOLE FOODS MARKET</t>
+          <t>COFFEE SHOP DOWNTOWN</t>
         </is>
       </c>
       <c r="E7">
-        <v>38.42</v>
+        <v>5.25</v>
       </c>
       <c r="F7"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Posted</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H7">
+        <v>1291.56</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8"/>
+      <c r="B8">
+        <v>45725</v>
+      </c>
+      <c r="C8"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>WHOLE FOODS MARKET</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>38.42</v>
+      </c>
+      <c r="F8"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="H8">
         <v>1296.81</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9"/>
     <row r="10"/>
     <row r="11"/>
@@ -250,6 +273,7 @@
     <row r="55"/>
     <row r="56"/>
     <row r="57"/>
+    <row r="58"/>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix import review bucket counts and refresh import rules list
Exclude other import sources from bank dedupe, classify transfers before
spending duplicate slots, detect E-PAYMENT from raw bank descriptions, and
render import rules immediately after confirm.

Co-authored-by: nixcapital <nixcapital@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/sample-bank.xlsx
+++ b/test/fixtures/sample-bank.xlsx
@@ -131,16 +131,16 @@
     <row r="5">
       <c r="A5"/>
       <c r="B5">
-        <v>45728</v>
+        <v>45729</v>
       </c>
       <c r="C5"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>STUDENT LOAN PAYMENT</t>
+          <t>XXXXXXXX        E-PAYMENT WEB 9999</t>
         </is>
       </c>
       <c r="E5">
-        <v>180</v>
+        <v>175.5</v>
       </c>
       <c r="F5"/>
       <c r="G5" t="inlineStr">
@@ -149,22 +149,22 @@
         </is>
       </c>
       <c r="H5">
-        <v>1279.56</v>
+        <v>854.06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6"/>
       <c r="B6">
-        <v>45727</v>
+        <v>45728</v>
       </c>
       <c r="C6"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Service Charge</t>
+          <t>STUDENT LOAN PAYMENT</t>
         </is>
       </c>
       <c r="E6">
-        <v>12</v>
+        <v>180</v>
       </c>
       <c r="F6"/>
       <c r="G6" t="inlineStr">
@@ -179,52 +179,75 @@
     <row r="7">
       <c r="A7"/>
       <c r="B7">
-        <v>45726</v>
+        <v>45727</v>
       </c>
       <c r="C7"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COFFEE SHOP DOWNTOWN</t>
+          <t>Service Charge</t>
         </is>
       </c>
       <c r="E7">
-        <v>5.25</v>
+        <v>12</v>
       </c>
       <c r="F7"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Posted</t>
         </is>
       </c>
       <c r="H7">
-        <v>1291.56</v>
+        <v>1279.56</v>
       </c>
     </row>
     <row r="8">
       <c r="A8"/>
       <c r="B8">
-        <v>45725</v>
+        <v>45726</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>WHOLE FOODS MARKET</t>
+          <t>COFFEE SHOP DOWNTOWN</t>
         </is>
       </c>
       <c r="E8">
-        <v>38.42</v>
+        <v>5.25</v>
       </c>
       <c r="F8"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Posted</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H8">
+        <v>1291.56</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9"/>
+      <c r="B9">
+        <v>45725</v>
+      </c>
+      <c r="C9"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>WHOLE FOODS MARKET</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>38.42</v>
+      </c>
+      <c r="F9"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="H9">
         <v>1296.81</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
@@ -274,6 +297,7 @@
     <row r="56"/>
     <row r="57"/>
     <row r="58"/>
+    <row r="59"/>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>